<commit_message>
docs(platform): record lan verification evidence
</commit_message>
<xml_diff>
--- a/docs/week2/05_第二周验收台账.xlsx
+++ b/docs/week2/05_第二周验收台账.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Rc62b2df854e2454a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A验收" sheetId="2" r:id="R73996b13a3f14676"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B验收" sheetId="3" r:id="R6efd25cc61674fa7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C验收" sheetId="4" r:id="R6c6f3ba127354399"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="协作交接" sheetId="5" r:id="R876ea38a596348af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="用户功能验收" sheetId="6" r:id="Rebf77bcbd6b54194"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20样本复评" sheetId="7" r:id="Rb264d946fcb943c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据索引" sheetId="8" r:id="R928ac8526b0d4759"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Rc40e654825d0487b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A验收" sheetId="2" r:id="Rf0651d3fff4f45e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B验收" sheetId="3" r:id="R35e483e685cd46c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C验收" sheetId="4" r:id="Rda23ce00507f43ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="协作交接" sheetId="5" r:id="R81af503100b046ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="用户功能验收" sheetId="6" r:id="R0230a3117064415a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20样本复评" sheetId="7" r:id="R54712443fac945e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据索引" sheetId="8" r:id="Raf0a52559a344bea"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -775,13 +775,13 @@
     <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="36" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="46" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="30" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="40" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -826,9 +826,11 @@
       <x:c r="C2" s="7" t="str">
         <x:v>LAN 另一设备首页/healthz/搜索/详情</x:v>
       </x:c>
-      <x:c r="D2" s="7" t="str"/>
+      <x:c r="D2" s="7" t="str">
+        <x:v>首页/搜索/healthz 截图已收；设备/详情/录屏待补</x:v>
+      </x:c>
       <x:c r="E2" s="7" t="str">
-        <x:v>evidence/week2/A/lan-device-*.png</x:v>
+        <x:v>evidence/week2/A/lan-home.png; lan-search.png; lan-healthz.png</x:v>
       </x:c>
       <x:c r="F2" s="7" t="str"/>
       <x:c r="G2" s="7" t="str"/>
@@ -837,7 +839,7 @@
       </x:c>
       <x:c r="I2" s="7" t="str">
         <x:f>IF(AND(D2&lt;&gt;"",E2&lt;&gt;"",F2&lt;&gt;"",G2&lt;&gt;"",H2=TRUE),"通过",IF(D2="","待填写",IF(E2="","缺证据",IF(OR(F2="",G2=""),"待接收","未达标"))))</x:f>
-        <x:v>待填写</x:v>
+        <x:v>待接收</x:v>
       </x:c>
       <x:c r="J2" s="7" t="str"/>
     </x:row>
@@ -3399,7 +3401,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
-        <x:v>evidence/week2/A/lan-device.png</x:v>
+        <x:v>evidence/week2/A/lan-home.png; lan-search.png; lan-healthz.png</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
         <x:v>截图</x:v>
@@ -3407,7 +3409,7 @@
       <x:c r="E2" s="7" t="str"/>
       <x:c r="F2" s="7" t="str"/>
       <x:c r="G2" s="7" t="str">
-        <x:v>待补</x:v>
+        <x:v>已收到，待补设备/时间</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
docs(week2): freeze auth/cas contract (4 roles + dev switch semantics)
</commit_message>
<xml_diff>
--- a/docs/week2/05_第二周验收台账.xlsx
+++ b/docs/week2/05_第二周验收台账.xlsx
@@ -956,7 +956,7 @@
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>首页/搜索/healthz 三张截图已收；访问设备：ASUS Vivobook S Flip（TN3604YA，Windows 11，192.168.43.110→组长机 192.168.43.50:5000）；访问时间 2026-09-19 20:36；详情页截图待补</t>
+          <t>首页/搜索/healthz 三张截图已收；访问设备：ASUS Vivobook S Flip（TN3604YA，Windows 11，192.168.43.110→LAN 服务 192.168.43.50:5000）；访问时间 2026-09-19 20:36；C 确认无需补详情页截图</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
@@ -964,8 +964,16 @@
           <t>evidence/week2/A/lan-home.png; lan-search.png; lan-healthz.png</t>
         </is>
       </c>
-      <c r="F2" s="8" t="str"/>
-      <c r="G2" s="8" t="str"/>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>3a34ea5（feat/week2-A-platform）</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>C 2026-09-21 确认接收（沟通记录，见 lan-verification.md）</t>
+        </is>
+      </c>
       <c r="H2" s="8" t="b">
         <v>0</v>
       </c>
@@ -993,15 +1001,19 @@
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>已覆盖测试</t>
+          <t>pytest 30/30 + 真实 HTTP 活体验证 4 场景全 PASS（开关关闭 404 / 6 种伪造 header 提权失败 / 开关显式开启才可用）</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>tests/core/test_api.py</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="str"/>
+          <t>evidence/week2/A/role-isolation-live.txt; role-isolation-test-output.txt; auth-contract.md; scripts/run_role_isolation.py</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>4fe2b69（feat/week2-A-platform）</t>
+        </is>
+      </c>
       <c r="G3" s="8" t="str"/>
       <c r="H3" s="8" t="b">
         <v>1</v>
@@ -3960,11 +3972,19 @@
           <t>截图</t>
         </is>
       </c>
-      <c r="E2" s="8" t="str"/>
-      <c r="F2" s="8" t="str"/>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>3a34ea5（feat/week2-A-platform）</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>C 2026-09-21 确认接收</t>
+        </is>
+      </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>设备/时间已补记（2026-09-21，见 lan-verification.md），详情页截图待补</t>
+          <t>已接收（C 2026-09-21，无需补详情页）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(week2): mark A-03 backup recovery as achieved (bb160a1)
</commit_message>
<xml_diff>
--- a/docs/week2/05_第二周验收台账.xlsx
+++ b/docs/week2/05_第二周验收台账.xlsx
@@ -1011,7 +1011,7 @@
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>4fe2b69（feat/week2-A-platform）</t>
+          <t>f88e52f06f（feat/week2-A-platform）</t>
         </is>
       </c>
       <c r="G3" s="8" t="str"/>
@@ -1040,22 +1040,31 @@
           <t>SQLite 备份恢复后三类行数一致</t>
         </is>
       </c>
-      <c r="D4" s="8" t="str"/>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>evidence/week2/A/backup-restore.json</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="str"/>
-      <c r="G4" s="8" t="str"/>
-      <c r="H4" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="I4" s="8">
-        <f>IF(AND(D4&lt;&gt;"",E4&lt;&gt;"",F4&lt;&gt;"",G4&lt;&gt;"",H4=TRUE),"通过",IF(D4="","待填写",IF(E4="","缺证据",IF(OR(F4="",G4=""),"待接收","未达标"))))</f>
-        <v/>
-      </c>
-      <c r="J4" s="8" t="str"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">data/app.db (5/7/11) → 模拟破坏 (3/4/5) → 恢复到 data/app-restored.db (5/7/11，SHA b343c3b4…077d076 与备份一致)；6 个敏感字段全 NULL、非敏感字段保留；篡改检测 exit=2、错误路径 exit=3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">evidence/week2/A/backup-recovery.md; _artifacts/step1-step6.txt</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bb160a1（feat/week2-A-platform）</t>
+        </is>
+      </c>
+      <c r="G4"/>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">禁字面量扫描 0 命中；A-03 验收项关闭，C 接收确认待补</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="1">
       <c r="A5" s="8" t="inlineStr">

</xml_diff>

<commit_message>
docs(week2): mark A-04 deployment as blocked (TCP/22 reach, auth-fail, 5 external gaps)
台账 A-04 行同步指向：
- D 列实际值：TCP/22 通 (RTT 11.7ms) / 80+443 拒绝 / SSH ubuntu+'lm@1215' 认证失败
- E 列证据路径：evidence/week2/A/deployment-precheck.md +
  progress/week2/A/deployment-blocker.md (9/24 升级版)
- F 列 commit: 3c953547b1ec（前置 9/24 阻塞收尾 commit）
- H 列指标达到目标: 0（阻塞，未达目标）
- J 列备注：A-04 阻塞；按任务书 §一不宣称上线；缺 5 项外部资源见 blocker.md §二
</commit_message>
<xml_diff>
--- a/docs/week2/05_第二周验收台账.xlsx
+++ b/docs/week2/05_第二周验收台账.xlsx
@@ -1082,26 +1082,31 @@
           <t>HTTPS/CAS 条件式结论</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>未提供服务器/域名/CAS</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>progress/week2/A/deployment-blocker.md</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="str"/>
-      <c r="G5" s="8" t="str"/>
-      <c r="H5" s="8" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" s="8">
-        <f>IF(AND(D5&lt;&gt;"",E5&lt;&gt;"",F5&lt;&gt;"",G5&lt;&gt;"",H5=TRUE),"通过",IF(D5="","待填写",IF(E5="","缺证据",IF(OR(F5="",G5=""),"待接收","未达标"))))</f>
-        <v/>
-      </c>
-      <c r="J5" s="8" t="str"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">81.70.40.146 TCP/22 通 (RTT 11.7ms) + 80/443 拒绝 + SSH ubuntu+lm@1215 认证失败（AuthenticationException）</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">evidence/week2/A/deployment-precheck.md; progress/week2/A/deployment-blocker.md (9/24 升级版)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3c953547b1ec (feat/week2-A-platform)</t>
+        </is>
+      </c>
+      <c r="G5"/>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A-04 阻塞；按任务书 §一不宣称上线；缺 5 项外部资源见 blocker.md §二</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="1">
       <c r="A6" s="8" t="n"/>

</xml_diff>